<commit_message>
Connected cardamom prices to API and Excel data
</commit_message>
<xml_diff>
--- a/Vrindavanam Glassmorphism/Vrindavanam/cardamom.xlsx
+++ b/Vrindavanam Glassmorphism/Vrindavanam/cardamom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Glassmorphism\Vrindavanam Glassmorphism\Vrindavanam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA957C6-AEDA-4821-96C9-41AEBBE1B9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD03ABE8-D541-4199-8C35-9BB4EA46282F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{213A37A3-F88C-42DF-B134-BBBC12CBE028}"/>
   </bookViews>
@@ -700,7 +700,7 @@
         <v>46171</v>
       </c>
       <c r="I2">
-        <v>550</v>
+        <v>700</v>
       </c>
       <c r="J2">
         <v>5</v>
@@ -715,7 +715,7 @@
         <v>34</v>
       </c>
       <c r="N2">
-        <v>2500</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -803,7 +803,7 @@
         <v>44</v>
       </c>
       <c r="N4">
-        <v>1750</v>
+        <v>9999</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>